<commit_message>
Regenerate dummy invoice files
</commit_message>
<xml_diff>
--- a/invoice_example.xlsx
+++ b/invoice_example.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>30 March 2026</t>
+          <t>04 September 2026</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>29 April 2026</t>
+          <t>04 October 2026</t>
         </is>
       </c>
     </row>

</xml_diff>